<commit_message>
Default Subtotal for not grouped .
</commit_message>
<xml_diff>
--- a/tests/Gauges/GroupTagTests_Simple_Empty.xlsx
+++ b/tests/Gauges/GroupTagTests_Simple_Empty.xlsx
@@ -322,7 +322,7 @@
       <x:diagonal/>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="25">
+  <x:cellStyleXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
@@ -351,16 +351,22 @@
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -384,20 +390,23 @@
     <x:xf numFmtId="4" fontId="0" fillId="3" borderId="6" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="4" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="4" fontId="12" fillId="3" borderId="4" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="4" fontId="12" fillId="3" borderId="4" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
     <x:xf numFmtId="17" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="75">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -542,22 +551,18 @@
       <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="1" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -594,7 +599,7 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -608,14 +613,6 @@
     </x:xf>
     <x:xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="1" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
@@ -1159,23 +1156,23 @@
       <x:c r="B6" s="38">
         <x:f>"632-1 Third Frydenhoj"&amp;" "&amp;""</x:f>
       </x:c>
-      <x:c r="C6" s="10"/>
-      <x:c r="D6" s="10"/>
-      <x:c r="E6" s="10"/>
-      <x:c r="F6" s="10"/>
+      <x:c r="C6" s="9"/>
+      <x:c r="D6" s="9"/>
+      <x:c r="E6" s="9"/>
+      <x:c r="F6" s="9"/>
       <x:c r="G6" s="10"/>
-      <x:c r="H6" s="56"/>
+      <x:c r="H6" s="11"/>
       <x:c r="I6" s="12"/>
       <x:c r="J6" s="13"/>
     </x:row>
     <x:row r="7" spans="1:10" ht="11.4" customHeight="1" x14ac:dyDescent="0.2">
-      <x:c r="B7" s="57"/>
-      <x:c r="C7" s="58"/>
-      <x:c r="D7" s="58"/>
-      <x:c r="E7" s="58"/>
-      <x:c r="F7" s="58"/>
+      <x:c r="B7" s="56"/>
+      <x:c r="C7" s="57"/>
+      <x:c r="D7" s="57"/>
+      <x:c r="E7" s="57"/>
+      <x:c r="F7" s="57"/>
       <x:c r="G7" s="58"/>
-      <x:c r="H7" s="57"/>
+      <x:c r="H7" s="56"/>
     </x:row>
     <x:row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <x:c r="B8" s="54" t="s">
@@ -1195,80 +1192,80 @@
       <x:c r="B9" s="41" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C9" s="10"/>
-      <x:c r="D9" s="10"/>
+      <x:c r="C9" s="9"/>
+      <x:c r="D9" s="9"/>
       <x:c r="E9" s="41" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="F9" s="59"/>
+      <x:c r="F9" s="16"/>
       <x:c r="G9" s="41" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="H9" s="59"/>
+      <x:c r="H9" s="16"/>
       <x:c r="I9" s="41" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="J9" s="59"/>
+      <x:c r="J9" s="16"/>
     </x:row>
     <x:row r="10" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <x:c r="B10" s="60"/>
-      <x:c r="C10" s="58"/>
-      <x:c r="D10" s="58"/>
-      <x:c r="E10" s="60"/>
-      <x:c r="F10" s="58"/>
-      <x:c r="G10" s="60"/>
-      <x:c r="H10" s="58"/>
-      <x:c r="I10" s="60"/>
-      <x:c r="J10" s="58"/>
+      <x:c r="B10" s="59"/>
+      <x:c r="C10" s="57"/>
+      <x:c r="D10" s="57"/>
+      <x:c r="E10" s="59"/>
+      <x:c r="F10" s="57"/>
+      <x:c r="G10" s="59"/>
+      <x:c r="H10" s="57"/>
+      <x:c r="I10" s="59"/>
+      <x:c r="J10" s="57"/>
     </x:row>
     <x:row r="11" spans="1:10" ht="20.4" customHeight="1" x14ac:dyDescent="0.2">
-      <x:c r="B11" s="61" t="s">
+      <x:c r="B11" s="60" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C11" s="62" t="s">
+      <x:c r="C11" s="61" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D11" s="61" t="s">
+      <x:c r="D11" s="60" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E11" s="61" t="s">
+      <x:c r="E11" s="60" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F11" s="61" t="s">
+      <x:c r="F11" s="60" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G11" s="63" t="s">
+      <x:c r="G11" s="62" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H11" s="64" t="s">
+      <x:c r="H11" s="63" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I11" s="64" t="s">
+      <x:c r="I11" s="63" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J11" s="64" t="s">
+      <x:c r="J11" s="63" t="s">
         <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:10" ht="10.2" customHeight="1" x14ac:dyDescent="0.2">
-      <x:c r="B12" s="65" t="s">
+      <x:c r="B12" s="64" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C12" s="66"/>
-      <x:c r="D12" s="67"/>
-      <x:c r="E12" s="66"/>
-      <x:c r="F12" s="68"/>
-      <x:c r="G12" s="69"/>
-      <x:c r="H12" s="70">
+      <x:c r="C12" s="65"/>
+      <x:c r="D12" s="66"/>
+      <x:c r="E12" s="65"/>
+      <x:c r="F12" s="67"/>
+      <x:c r="G12" s="68"/>
+      <x:c r="H12" s="69">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I12" s="71"/>
-      <x:c r="J12" s="70">
-        <x:v>0</x:v>
+      <x:c r="I12" s="70"/>
+      <x:c r="J12" s="69">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <x:c r="C13" s="72"/>
+      <x:c r="C13" s="71"/>
       <x:c r="G13" s="53"/>
     </x:row>
     <x:row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1280,15 +1277,15 @@
       </x:c>
     </x:row>
     <x:row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <x:c r="B15" s="73" t="s">
+      <x:c r="B15" s="46" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="C15" s="10"/>
-      <x:c r="D15" s="10"/>
-      <x:c r="E15" s="73" t="s">
+      <x:c r="C15" s="9"/>
+      <x:c r="D15" s="9"/>
+      <x:c r="E15" s="46" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="F15" s="74"/>
+      <x:c r="F15" s="17"/>
     </x:row>
     <x:row r="16" ht="11.4" customHeight="1" x14ac:dyDescent="0.2"/>
   </x:sheetData>

</xml_diff>